<commit_message>
These are so many updates to plotting and analysis
</commit_message>
<xml_diff>
--- a/_test_P111zero.xlsx
+++ b/_test_P111zero.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bgulick\Downloads\vCIJ_tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D8452F-EA75-4A79-AAD9-86F6F50DA857}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72999D97-DE89-419C-92D9-43C6000886CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AF17594D-297A-453C-A603-553966F3F3E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{AF17594D-297A-453C-A603-553966F3F3E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="24" r:id="rId1"/>
@@ -23289,6 +23289,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="40.7109375" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>